<commit_message>
feat: add temporary Guild menu client screen with navigation and server interactions
</commit_message>
<xml_diff>
--- a/docs/CTRBLXAI_Build_Plan.xlsx
+++ b/docs/CTRBLXAI_Build_Plan.xlsx
@@ -9067,7 +9067,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -9185,7 +9184,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -10192,7 +10190,6 @@
         </is>
       </c>
     </row>
-    <row r="48"/>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
@@ -10242,7 +10239,6 @@
         </is>
       </c>
     </row>
-    <row r="56"/>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
@@ -10264,7 +10260,6 @@
         </is>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
@@ -10357,7 +10352,6 @@
         </is>
       </c>
     </row>
-    <row r="67"/>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
@@ -10585,7 +10579,6 @@
         </is>
       </c>
     </row>
-    <row r="79"/>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
@@ -10653,7 +10646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -10666,497 +10659,668 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>02 — Service Boundaries</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Owns</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Reads</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Writes</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Must_Not_Own</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Primary_Interface</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Failure_Boundary</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Authoritative implementation boundary map. Services communicate through explicit commands, events, IDs, and immutable snapshots.</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Battle Coordinator</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Battle lifecycle, phase, CT advancement, ready-unit arbitration</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Battle state, scheduled events</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Phase, CT, active command gate</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Skill formulas, reward tables</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>AdvanceClock, BeginTurn, EndTurn</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Reject advancement while command/event resolution is open</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Command Service</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Player/AI command envelope and validation orchestration</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Actor state, loadout, selected target</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Committed command or failure result</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Damage math or effect behavior</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>ValidateAndCommit(Command)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>No partial resource payment on failed commitment</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>System</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>Owns</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>Reads</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>Writes</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>Must Not Own</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>Primary Interface</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>Failure Boundary</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Targeting Service</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Selection legality and candidate enumeration</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Map, units, Skill target metadata</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Target lock, anchor, candidate set</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Damage/effect resolution</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ValidateSelection, EnumerateCandidates</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Returns reason-coded invalid result</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Battle Coordinator</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Battle lifecycle, phase, CT advancement, ready-unit arbitration</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Battle state, scheduled events</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>Phase, CT, active command gate</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>Skill formulas, reward tables</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>AdvanceClock, BeginTurn, EndTurn</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Reject advancement while command/event resolution is open</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Skill Service</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Skill lifecycle and authored Skill snapshot</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Skill catalog, actor, weapon, Augments</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SkillResolutionContext</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Reward generation</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>CommitSkill, ActivateSkill</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>One context per execution; immutable after commitment</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Command Service</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Player/AI command envelope and validation orchestration</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Actor state, loadout, selected target</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>Committed command or failure result</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>Damage math or effect behavior</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>ValidateAndCommit(Command)</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>No partial resource payment on failed commitment</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Combat Resolver</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Primary numerical effect resolution</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Resolution context, target state</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Damage/heal/shield/effect outcomes</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Event queue scheduling policy</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>ResolvePrimaryEffect</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>No direct recursive trigger calls</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Targeting Service</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Selection legality and candidate enumeration</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Map, units, Skill target metadata</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Target lock, anchor, candidate set</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>Damage/effect resolution</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>ValidateSelection, EnumerateCandidates</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Returns reason-coded invalid result</t>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Trigger Service</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Eligibility, caps, processed sets, event production</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Outcomes, trigger subscriptions, turn counters</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Queued secondary events</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Primary formula evaluation</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>EvaluateTriggers, Enqueue</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Every repeat has a finite cap or processed set</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Skill Service</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Skill lifecycle and authored Skill snapshot</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Skill catalog, actor, weapon, Augments</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>SkillResolutionContext</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>Reward generation</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>CommitSkill, ActivateSkill</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>One context per execution; immutable after commitment</t>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Status Service</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Status instances, duration, stacks, ticks</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Source snapshot, target, clock</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Status state and scheduled ticks</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Skill attachment state</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>ApplyStatus, TickStatus, RemoveStatus</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Stable order; no same-event recursive evolution</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Combat Resolver</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Primary numerical effect resolution</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Resolution context, target state</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Damage/heal/shield/effect outcomes</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>Event queue scheduling policy</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>ResolvePrimaryEffect</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>No direct recursive trigger calls</t>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Summon Service</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Summon creation, ownership, replacement, intrinsic profile</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Summon Skill context, tile, owner snapshot</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Unit runtime entity</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Doctrine/loot eligibility by default</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>CreateSummon, ReplaceOwnedSummon</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Invalid spawn fails without deleting existing summon</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Trigger Service</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Eligibility, caps, processed sets, event production</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>Outcomes, trigger subscriptions, turn counters</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Queued secondary events</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>Primary formula evaluation</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>EvaluateTriggers, Enqueue</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Every repeat has a finite cap or processed set</t>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Equipment Service</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Equipped state, hand legality, reduced-use profiles, Break-dependent activation</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Loadout, Race/Doctrine enablement</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Active equipment profile</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Skill authored inheritance values</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>ValidateLoadout, RecomputeActiveProfile</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Atomic hand-state transition</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Status Service</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>Status instances, duration, stacks, ticks</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>Source snapshot, target, clock</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>Status state and scheduled ticks</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>Skill attachment state</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>ApplyStatus, TickStatus, RemoveStatus</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>Stable order; no same-event recursive evolution</t>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Reward Service</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Reward opportunity through generated reward</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Source, Fortune snapshot, eligibility tables</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Reward result and audit trail</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Combat damage or KO qualification</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>GenerateReward(Opportunity)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Zero-weight and ineligible categories remain impossible</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Summon Service</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Summon creation, ownership, replacement, intrinsic profile</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>Summon Skill context, tile, owner snapshot</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>Unit runtime entity</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>Doctrine/loot eligibility by default</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>CreateSummon, ReplaceOwnedSummon</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Invalid spawn fails without deleting existing summon</t>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Persistence Service</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Save/load, schema version, migration, referential validation</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Persistent entities</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Serialized state / load result</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Transient event queue unless combat-save enabled</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Save, Load, Migrate</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Load fails safely with diagnostics; never invent missing content</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Equipment Service</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Equipped state, hand legality, reduced-use profiles, Break-dependent activation</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>Loadout, Race/Doctrine enablement</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>Active equipment profile</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>Skill authored inheritance values</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>ValidateLoadout, RecomputeActiveProfile</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>Atomic hand-state transition</t>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Map Service</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Runtime map graph, tile/object/effect state, connectivity</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Biome/region/template definitions, generation seed</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Tile state, object state, effect state</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Combat formulas, reward tables, unit stats</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>GenerateMap, ValidateConnectivity, GetTileState</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Invalid generation retries bounded; falls back to safe template</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Reward Service</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Reward opportunity through generated reward</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>Source, Fortune snapshot, eligibility tables</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>Reward result and audit trail</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>Combat damage or KO qualification</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>GenerateReward(Opportunity)</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>Zero-weight and ineligible categories remain impossible</t>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Recruitment Service</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Recruit pool generation, hire eligibility, hire cost resolution</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Guild level, recruitment costs (economy_framework), roster capacity, region/unlock gates</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Hire request -&gt; new unit handed to Persistence Service for recording</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Unit storage/roster persistence, combat, loot generation</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>GenerateRecruitPool, ValidateHire, CommitHire</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>No gold charged on failed hire (insufficient gold / roster full); pool reroll bounded</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Persistence Service</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>Save/load, schema version, migration, referential validation</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>Persistent entities</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>Serialized state / load result</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>Transient event queue unless combat-save enabled</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>Save, Load, Migrate</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>Load fails safely with diagnostics; never invent missing content</t>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Guild Service</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Account-wide Guild level and Guild XP accrual, unlock gating</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Completed battles/quests, Guild XP rules (loot_progression), content level for trivial-reduction bands</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Guild XP delta, Guild level, unlock state</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Unit combat stats, loot rarity, Expedition Fortune (locked exclusions)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>AwardGuildXp, GetUnlocks, GetGuildLevel</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Guild XP never per-kill; trivial content reduced via unit-XP gap bands; no stat/loot effect</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Map Service</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Runtime map graph, tile/object/effect state, connectivity</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>Biome/region/template definitions, generation seed</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>Tile state, object state, effect state</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>Combat formulas, reward tables, unit stats</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>GenerateMap, ValidateConnectivity, GetTileState</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>Invalid generation retries bounded; falls back to safe template</t>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Blacksmith Service</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Equipment upgrade/downgrade transaction (level change, rarity bonus budget recompute)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Target item, upgrade gold cost formula + material recipes (economy_framework/materials_system), player gold/materials</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Modified item handed to Persistence Service; gold+materials debited</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>New item generation, loot tables, combat</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>ValidateUpgrade, CommitUpgrade, CommitDowngrade</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Atomic: gold+materials charged only on success; downgrade is free (no compensation); never creates a new item</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Currency Service</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Player gold balance and 5 material tier counters (T1-T5); atomic credit/debit transactions</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>economy_framework (gold sources/sinks), materials_system (counters, drop grants), save_data_contract Key 2</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Updated gold + material counts handed to Persistence Service (DataStore Key 2 — Inventory + Currencies)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Reward generation, item generation, combat, pricing formulas (reads prices, does not define them)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>GetBalance, CanAfford, Credit, Debit (atomic multi-cost)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Debit is all-or-nothing: insufficient gold OR materials cancels the whole charge, no partial spend; balance never negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Progression Service</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Unit XP accrual, distribution, level-up, and the unit-XP grant sink the battle/dispatch/explore systems call</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>unit_progression (kill XP, level curve, distribution rates, overleveled bands, Human +10%), race growth rates, battle result (kills, objectives, deployed/benched/KO sets)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Updated unit XP + level handed to Persistence Service (DataStore Key 1/3); level-up events for presentation</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Combat damage math, reward/loot generation, Guild XP (that is Guild Service), equipment stats</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>AwardBattleXp, GrantUnitXp, GetUnitLevelProgress</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>XP never granted twice for the same source; level clamps at 99; benched 65% / KO-on-win full / deployed 100% applied exactly once</t>
         </is>
       </c>
     </row>

</xml_diff>